<commit_message>
fix: robust JSON extraction and corrected page maps for all 4 insurers
- Replace brittle fence-stripping cleanup with {[^{}]*} regex: extracts the
  first flat JSON object, immune to prose-before-fence and prose-after-fence
  patterns that caused 5 parse failures per run
- ASR: solvency pages corrected to p406 (EOF 12,618 / SCR 5,743 / 220%);
  insurance_svc_result extended to p289-292 for CSM/RA release detail;
  GWP pages extended to include segment P&L pages
- NN Group: portfolio_overview/gross_premium add p221-222 (GWP Life 8,787 /
  Non-life 4,469); investments_note corrected to p173-176 (FVTPL 56,570)
- Athora: gross_premium pages reordered to prioritise p81 (insurance revenue 2,110)
- GWP prompt updated to fall back to insurance revenue when GWP not available

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/All_Insurers_2025_Databook.xlsx
+++ b/All_Insurers_2025_Databook.xlsx
@@ -1510,7 +1510,7 @@
         <v>70</v>
       </c>
       <c r="B102" t="n">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="C102" t="s">
         <v>8</v>
@@ -2479,7 +2479,7 @@
         <v>36</v>
       </c>
       <c r="B60" t="n">
-        <v>0.0058</v>
+        <v>0.0265</v>
       </c>
       <c r="C60" t="s">
         <v>37</v>
@@ -2490,7 +2490,7 @@
         <v>38</v>
       </c>
       <c r="B61" t="n">
-        <v>0.0058</v>
+        <v>0.0305</v>
       </c>
       <c r="C61" t="s">
         <v>37</v>
@@ -2501,7 +2501,7 @@
         <v>39</v>
       </c>
       <c r="B62" t="n">
-        <v>0.0058</v>
+        <v>0.0343</v>
       </c>
       <c r="C62" t="s">
         <v>37</v>
@@ -2521,7 +2521,7 @@
         <v>41</v>
       </c>
       <c r="B64" t="n">
-        <v>0.0058</v>
+        <v>0.0378</v>
       </c>
       <c r="C64" t="s">
         <v>37</v>
@@ -2532,7 +2532,7 @@
         <v>42</v>
       </c>
       <c r="B65" t="n">
-        <v>0.0049</v>
+        <v>0.0368</v>
       </c>
       <c r="C65" t="s">
         <v>37</v>
@@ -2543,7 +2543,7 @@
         <v>43</v>
       </c>
       <c r="B66" t="n">
-        <v>0.0031</v>
+        <v>0.0349</v>
       </c>
       <c r="C66" t="s">
         <v>37</v>
@@ -2628,7 +2628,9 @@
       <c r="A80" t="s">
         <v>55</v>
       </c>
-      <c r="B80"/>
+      <c r="B80" t="n">
+        <v>4122</v>
+      </c>
       <c r="C80" t="s">
         <v>8</v>
       </c>
@@ -2637,7 +2639,9 @@
       <c r="A81" t="s">
         <v>56</v>
       </c>
-      <c r="B81"/>
+      <c r="B81" t="n">
+        <v>117</v>
+      </c>
       <c r="C81" t="s">
         <v>8</v>
       </c>
@@ -2646,7 +2650,9 @@
       <c r="A82" t="s">
         <v>57</v>
       </c>
-      <c r="B82"/>
+      <c r="B82" t="n">
+        <v>111</v>
+      </c>
       <c r="C82" t="s">
         <v>8</v>
       </c>
@@ -2655,7 +2661,9 @@
       <c r="A83" t="s">
         <v>58</v>
       </c>
-      <c r="B83"/>
+      <c r="B83" t="n">
+        <v>470</v>
+      </c>
       <c r="C83" t="s">
         <v>8</v>
       </c>
@@ -2664,7 +2672,9 @@
       <c r="A84" t="s">
         <v>59</v>
       </c>
-      <c r="B84"/>
+      <c r="B84" t="n">
+        <v>-266</v>
+      </c>
       <c r="C84" t="s">
         <v>8</v>
       </c>
@@ -2673,7 +2683,9 @@
       <c r="A85" t="s">
         <v>60</v>
       </c>
-      <c r="B85"/>
+      <c r="B85" t="n">
+        <v>14</v>
+      </c>
       <c r="C85" t="s">
         <v>8</v>
       </c>
@@ -2682,7 +2694,9 @@
       <c r="A86" t="s">
         <v>61</v>
       </c>
-      <c r="B86"/>
+      <c r="B86" t="n">
+        <v>4568</v>
+      </c>
       <c r="C86" t="s">
         <v>8</v>
       </c>
@@ -3111,7 +3125,7 @@
         <v>100</v>
       </c>
       <c r="B144" t="n">
-        <v>2.18</v>
+        <v>2.2</v>
       </c>
       <c r="C144" t="s">
         <v>101</v>
@@ -3130,7 +3144,9 @@
       <c r="A146" t="s">
         <v>103</v>
       </c>
-      <c r="B146"/>
+      <c r="B146" t="n">
+        <v>5743</v>
+      </c>
       <c r="C146" t="s">
         <v>101</v>
       </c>
@@ -3139,7 +3155,9 @@
       <c r="A147" t="s">
         <v>104</v>
       </c>
-      <c r="B147"/>
+      <c r="B147" t="n">
+        <v>12618</v>
+      </c>
       <c r="C147" t="s">
         <v>101</v>
       </c>
@@ -3148,9 +3166,7 @@
       <c r="A148" t="s">
         <v>105</v>
       </c>
-      <c r="B148" t="n">
-        <v>1315</v>
-      </c>
+      <c r="B148"/>
       <c r="C148" t="s">
         <v>101</v>
       </c>
@@ -3516,7 +3532,9 @@
       <c r="A25" t="s">
         <v>10</v>
       </c>
-      <c r="B25"/>
+      <c r="B25" t="n">
+        <v>2696</v>
+      </c>
       <c r="C25" t="s">
         <v>12</v>
       </c>
@@ -3525,7 +3543,9 @@
       <c r="A26" t="s">
         <v>18</v>
       </c>
-      <c r="B26"/>
+      <c r="B26" t="n">
+        <v>140460</v>
+      </c>
       <c r="C26" t="s">
         <v>12</v>
       </c>
@@ -4463,7 +4483,9 @@
       <c r="A156" t="s">
         <v>111</v>
       </c>
-      <c r="B156"/>
+      <c r="B156" t="n">
+        <v>22374</v>
+      </c>
       <c r="C156" t="s">
         <v>108</v>
       </c>
@@ -4481,9 +4503,7 @@
       <c r="A158" t="s">
         <v>113</v>
       </c>
-      <c r="B158" t="n">
-        <v>-3030</v>
-      </c>
+      <c r="B158"/>
       <c r="C158" t="s">
         <v>108</v>
       </c>
@@ -4501,9 +4521,7 @@
       <c r="A160" t="s">
         <v>18</v>
       </c>
-      <c r="B160" t="n">
-        <v>196455</v>
-      </c>
+      <c r="B160"/>
       <c r="C160" t="s">
         <v>12</v>
       </c>
@@ -4550,7 +4568,9 @@
       <c r="A169" t="s">
         <v>118</v>
       </c>
-      <c r="B169"/>
+      <c r="B169" t="n">
+        <v>8787</v>
+      </c>
       <c r="C169" t="s">
         <v>119</v>
       </c>
@@ -4568,7 +4588,9 @@
       <c r="A171" t="s">
         <v>121</v>
       </c>
-      <c r="B171"/>
+      <c r="B171" t="n">
+        <v>4469</v>
+      </c>
       <c r="C171" t="s">
         <v>119</v>
       </c>
@@ -4595,7 +4617,9 @@
       <c r="A174" t="s">
         <v>18</v>
       </c>
-      <c r="B174"/>
+      <c r="B174" t="n">
+        <v>13256</v>
+      </c>
       <c r="C174" t="s">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
fix(asr): correct page references for insurance service result, CSM maturity, and discount rate labels
- insurance_svc_result: p289-292 (accounting policy) → p347-348 (section 7.6.1 with
  CSM release, RA release, and insurance revenue breakdown by segment)
- csm_maturity: p323-324 (GMM component tables) → p332 (GMM maturity, section 7.5.13.6)
  + p339 (VFA maturity, section 7.5.14.3)
- disc_liquid_label: "liquid risk-free" → "0% (min)" (actual table row label on p330)
- disc_illiquid_label: "illiquidity premium added" → "100% (max)" (actual table row label)
- net_financial_result: p290-291 → p350 (section 7.6.7 investment & finance result)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/All_Insurers_2025_Databook.xlsx
+++ b/All_Insurers_2025_Databook.xlsx
@@ -1543,9 +1543,7 @@
       <c r="A105" t="s">
         <v>72</v>
       </c>
-      <c r="B105" t="n">
-        <v>306</v>
-      </c>
+      <c r="B105"/>
       <c r="C105" t="s">
         <v>8</v>
       </c>
@@ -1554,9 +1552,7 @@
       <c r="A106" t="s">
         <v>73</v>
       </c>
-      <c r="B106" t="n">
-        <v>533</v>
-      </c>
+      <c r="B106"/>
       <c r="C106" t="s">
         <v>8</v>
       </c>
@@ -1954,7 +1950,7 @@
         <v>113</v>
       </c>
       <c r="B159" t="n">
-        <v>5005</v>
+        <v>5049</v>
       </c>
       <c r="C159" t="s">
         <v>109</v>
@@ -2324,7 +2320,9 @@
       <c r="A34" t="s">
         <v>23</v>
       </c>
-      <c r="B34"/>
+      <c r="B34" t="n">
+        <v>466</v>
+      </c>
       <c r="C34" t="s">
         <v>24</v>
       </c>
@@ -2333,7 +2331,9 @@
       <c r="A35" t="s">
         <v>25</v>
       </c>
-      <c r="B35"/>
+      <c r="B35" t="n">
+        <v>191</v>
+      </c>
       <c r="C35" t="s">
         <v>24</v>
       </c>
@@ -2342,7 +2342,9 @@
       <c r="A36" t="s">
         <v>26</v>
       </c>
-      <c r="B36"/>
+      <c r="B36" t="n">
+        <v>3918</v>
+      </c>
       <c r="C36" t="s">
         <v>24</v>
       </c>
@@ -2423,7 +2425,9 @@
       <c r="A51" t="s">
         <v>36</v>
       </c>
-      <c r="B51"/>
+      <c r="B51" t="n">
+        <v>0.0207</v>
+      </c>
       <c r="C51" t="s">
         <v>37</v>
       </c>
@@ -2432,7 +2436,9 @@
       <c r="A52" t="s">
         <v>38</v>
       </c>
-      <c r="B52"/>
+      <c r="B52" t="n">
+        <v>0.0247</v>
+      </c>
       <c r="C52" t="s">
         <v>37</v>
       </c>
@@ -2441,7 +2447,9 @@
       <c r="A53" t="s">
         <v>39</v>
       </c>
-      <c r="B53"/>
+      <c r="B53" t="n">
+        <v>0.0285</v>
+      </c>
       <c r="C53" t="s">
         <v>37</v>
       </c>
@@ -2459,7 +2467,9 @@
       <c r="A55" t="s">
         <v>41</v>
       </c>
-      <c r="B55"/>
+      <c r="B55" t="n">
+        <v>0.032</v>
+      </c>
       <c r="C55" t="s">
         <v>37</v>
       </c>
@@ -2468,7 +2478,9 @@
       <c r="A56" t="s">
         <v>42</v>
       </c>
-      <c r="B56"/>
+      <c r="B56" t="n">
+        <v>0.0319</v>
+      </c>
       <c r="C56" t="s">
         <v>37</v>
       </c>
@@ -2477,7 +2489,9 @@
       <c r="A57" t="s">
         <v>43</v>
       </c>
-      <c r="B57"/>
+      <c r="B57" t="n">
+        <v>0.0318</v>
+      </c>
       <c r="C57" t="s">
         <v>37</v>
       </c>
@@ -2486,7 +2500,9 @@
       <c r="A58" t="s">
         <v>44</v>
       </c>
-      <c r="B58"/>
+      <c r="B58" t="n">
+        <v>0.0318</v>
+      </c>
       <c r="C58" t="s">
         <v>37</v>
       </c>
@@ -2500,7 +2516,9 @@
       <c r="A61" t="s">
         <v>36</v>
       </c>
-      <c r="B61"/>
+      <c r="B61" t="n">
+        <v>0.0265</v>
+      </c>
       <c r="C61" t="s">
         <v>37</v>
       </c>
@@ -2509,7 +2527,9 @@
       <c r="A62" t="s">
         <v>38</v>
       </c>
-      <c r="B62"/>
+      <c r="B62" t="n">
+        <v>0.0305</v>
+      </c>
       <c r="C62" t="s">
         <v>37</v>
       </c>
@@ -2518,7 +2538,9 @@
       <c r="A63" t="s">
         <v>39</v>
       </c>
-      <c r="B63"/>
+      <c r="B63" t="n">
+        <v>0.0343</v>
+      </c>
       <c r="C63" t="s">
         <v>37</v>
       </c>
@@ -2536,7 +2558,9 @@
       <c r="A65" t="s">
         <v>41</v>
       </c>
-      <c r="B65"/>
+      <c r="B65" t="n">
+        <v>0.0378</v>
+      </c>
       <c r="C65" t="s">
         <v>37</v>
       </c>
@@ -2545,7 +2569,9 @@
       <c r="A66" t="s">
         <v>42</v>
       </c>
-      <c r="B66"/>
+      <c r="B66" t="n">
+        <v>0.0368</v>
+      </c>
       <c r="C66" t="s">
         <v>37</v>
       </c>
@@ -2554,7 +2580,9 @@
       <c r="A67" t="s">
         <v>43</v>
       </c>
-      <c r="B67"/>
+      <c r="B67" t="n">
+        <v>0.0357</v>
+      </c>
       <c r="C67" t="s">
         <v>37</v>
       </c>
@@ -2563,7 +2591,9 @@
       <c r="A68" t="s">
         <v>44</v>
       </c>
-      <c r="B68"/>
+      <c r="B68" t="n">
+        <v>0.0349</v>
+      </c>
       <c r="C68" t="s">
         <v>37</v>
       </c>
@@ -2827,7 +2857,9 @@
       <c r="A103" t="s">
         <v>70</v>
       </c>
-      <c r="B103"/>
+      <c r="B103" t="n">
+        <v>297</v>
+      </c>
       <c r="C103" t="s">
         <v>8</v>
       </c>
@@ -2836,7 +2868,9 @@
       <c r="A104" t="s">
         <v>71</v>
       </c>
-      <c r="B104"/>
+      <c r="B104" t="n">
+        <v>933</v>
+      </c>
       <c r="C104" t="s">
         <v>8</v>
       </c>
@@ -2845,7 +2879,9 @@
       <c r="A105" t="s">
         <v>72</v>
       </c>
-      <c r="B105"/>
+      <c r="B105" t="n">
+        <v>919</v>
+      </c>
       <c r="C105" t="s">
         <v>8</v>
       </c>
@@ -2854,7 +2890,9 @@
       <c r="A106" t="s">
         <v>73</v>
       </c>
-      <c r="B106"/>
+      <c r="B106" t="n">
+        <v>2627</v>
+      </c>
       <c r="C106" t="s">
         <v>8</v>
       </c>
@@ -2863,7 +2901,9 @@
       <c r="A107" t="s">
         <v>74</v>
       </c>
-      <c r="B107"/>
+      <c r="B107" t="n">
+        <v>4774</v>
+      </c>
       <c r="C107" t="s">
         <v>12</v>
       </c>
@@ -3061,9 +3101,7 @@
       <c r="A132" t="s">
         <v>91</v>
       </c>
-      <c r="B132" t="n">
-        <v>3</v>
-      </c>
+      <c r="B132"/>
       <c r="C132" t="s">
         <v>8</v>
       </c>
@@ -3072,9 +3110,7 @@
       <c r="A133" t="s">
         <v>92</v>
       </c>
-      <c r="B133" t="n">
-        <v>6</v>
-      </c>
+      <c r="B133"/>
       <c r="C133" t="s">
         <v>8</v>
       </c>

</xml_diff>